<commit_message>
feat(client-data): 💄 Sync dukestrategies overlay — brand realignment
Brand re-encode from client-data 0d3c8fb: dark #222222 primary, coral
demoted to accent, dark photo overlay, rebuilt chart palettes, new
images/manifest.json with per-image overlay policies, guidelines v1.1.
Renders via stromy-format pick this up at call time — no MCP redeploy.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/companies/dukestrategies/dukestrategies-client-data-overview.xlsx
+++ b/companies/dukestrategies/dukestrategies-client-data-overview.xlsx
@@ -34,13 +34,13 @@
     <font>
       <name val="Century Gothic"/>
       <b val="1"/>
-      <color rgb="00FF7F66"/>
+      <color rgb="00222222"/>
       <sz val="18"/>
     </font>
     <font>
       <name val="Century Gothic"/>
       <i val="1"/>
-      <color rgb="00F47E6C"/>
+      <color rgb="00FF7F66"/>
       <sz val="12"/>
     </font>
     <font>
@@ -52,18 +52,18 @@
     <font>
       <name val="Century Gothic"/>
       <b val="1"/>
-      <color rgb="00FF7F66"/>
+      <color rgb="00222222"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Century Gothic"/>
-      <color rgb="00807F83"/>
+      <color rgb="003A393C"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Century Gothic"/>
       <i val="1"/>
-      <color rgb="00DFDFE0"/>
+      <color rgb="00807F83"/>
       <sz val="8"/>
     </font>
     <font>
@@ -74,17 +74,17 @@
     </font>
     <font>
       <name val="Century Gothic"/>
-      <color rgb="00807F83"/>
+      <color rgb="003A393C"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Century Gothic"/>
       <b val="1"/>
-      <color rgb="00FF7F66"/>
+      <color rgb="00222222"/>
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="13">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -93,12 +93,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DFDFE0"/>
+        <fgColor rgb="005A595C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FF7F66"/>
+        <fgColor rgb="00222222"/>
       </patternFill>
     </fill>
     <fill>
@@ -113,7 +113,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F47E6C"/>
+        <fgColor rgb="00FF7F66"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="003A393C"/>
       </patternFill>
     </fill>
     <fill>
@@ -123,22 +128,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="004CAF50"/>
+        <fgColor rgb="005B9A6B"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC107"/>
+        <fgColor rgb="00D4A544"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DC3545"/>
+        <fgColor rgb="00C4544A"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EE5536"/>
+        <fgColor rgb="00E86B54"/>
       </patternFill>
     </fill>
     <fill>
@@ -159,7 +164,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -210,12 +215,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -731,7 +737,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>118</t>
+          <t>126</t>
         </is>
       </c>
     </row>
@@ -767,7 +773,7 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>81</t>
+          <t>82</t>
         </is>
       </c>
     </row>
@@ -791,7 +797,7 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>6</t>
         </is>
       </c>
     </row>
@@ -821,7 +827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F127"/>
+  <dimension ref="A1:F135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1141,7 +1147,7 @@
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>6.5 KB</t>
+          <t>8.7 KB</t>
         </is>
       </c>
       <c r="E14" s="12" t="inlineStr">
@@ -1153,7 +1159,7 @@
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>guidelines.md</t>
+          <t>dukestrategies-client-data-overview.xlsx</t>
         </is>
       </c>
       <c r="B15" s="9" t="inlineStr">
@@ -1163,213 +1169,213 @@
       </c>
       <c r="C15" s="9" t="inlineStr">
         <is>
-          <t>Markdown</t>
+          <t>XLSX</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>14.0 KB</t>
+          <t>18.5 KB</t>
         </is>
       </c>
       <c r="E15" s="10" t="inlineStr">
         <is>
-          <t>Brand usage guidelines</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>images/Erasmusbrug_zwart.jpg</t>
+          <t>fonts/Montserrat-Italic[wght].ttf</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>fonts</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>Font TTF</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>1135.1 KB</t>
+          <t>744.5 KB</t>
         </is>
       </c>
       <c r="E16" s="12" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>Font file — Montserrat-Italic[wght]</t>
         </is>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>images/Nesciobrug.jpg</t>
+          <t>fonts/Montserrat[wght].ttf</t>
         </is>
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>fonts</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>Font TTF</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
         <is>
-          <t>1168.7 KB</t>
+          <t>727.5 KB</t>
         </is>
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>Font file — Montserrat[wght]</t>
         </is>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>images/Pythonbrug_Amsterdam_contrast.jpg</t>
+          <t>fonts/OFL-Montserrat.txt</t>
         </is>
       </c>
       <c r="B18" s="11" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>fonts</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>588.3 KB</t>
+          <t>4.3 KB</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>Font file — OFL-Montserrat</t>
         </is>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>images/bridge-architecture-bw-lines.jpg</t>
+          <t>fonts/OFL-SpaceMono.txt</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>fonts</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>Text</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>1303.2 KB</t>
+          <t>4.3 KB</t>
         </is>
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>Font file — OFL-SpaceMono</t>
         </is>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="11" t="inlineStr">
         <is>
-          <t>images/bridge-fog-water-minimalist.jpg</t>
+          <t>fonts/SpaceMono-Bold.ttf</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>fonts</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>Font TTF</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>1629.4 KB</t>
+          <t>95.9 KB</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>Font file — SpaceMono-Bold</t>
         </is>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>images/brooklyn-bridge-bw.jpg</t>
+          <t>fonts/SpaceMono-Regular.ttf</t>
         </is>
       </c>
       <c r="B21" s="9" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>fonts</t>
         </is>
       </c>
       <c r="C21" s="9" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>Font TTF</t>
         </is>
       </c>
       <c r="D21" s="9" t="inlineStr">
         <is>
-          <t>4581.0 KB</t>
+          <t>97.0 KB</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>Font file — SpaceMono-Regular</t>
         </is>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>images/cable-bridge-dark-sky-dramatic.jpg</t>
+          <t>guidelines.md</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>images</t>
+          <t>root</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>Markdown</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>612.4 KB</t>
+          <t>15.8 KB</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr">
         <is>
-          <t>Photography / imagery asset</t>
+          <t>Brand usage guidelines</t>
         </is>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>images/cable-bridge-geometric-perspective.jpg</t>
+          <t>images/Erasmusbrug_zwart.jpg</t>
         </is>
       </c>
       <c r="B23" s="9" t="inlineStr">
@@ -1384,7 +1390,7 @@
       </c>
       <c r="D23" s="9" t="inlineStr">
         <is>
-          <t>1287.9 KB</t>
+          <t>1135.1 KB</t>
         </is>
       </c>
       <c r="E23" s="10" t="inlineStr">
@@ -1396,7 +1402,7 @@
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="11" t="inlineStr">
         <is>
-          <t>images/cable-bridge-golden-hour.jpg</t>
+          <t>images/Nesciobrug.jpg</t>
         </is>
       </c>
       <c r="B24" s="11" t="inlineStr">
@@ -1411,7 +1417,7 @@
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>2521.7 KB</t>
+          <t>1168.7 KB</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
@@ -1423,7 +1429,7 @@
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>images/cable-bridge-grayscale-dramatic.jpg</t>
+          <t>images/Pythonbrug_Amsterdam_contrast.jpg</t>
         </is>
       </c>
       <c r="B25" s="9" t="inlineStr">
@@ -1438,7 +1444,7 @@
       </c>
       <c r="D25" s="9" t="inlineStr">
         <is>
-          <t>1669.8 KB</t>
+          <t>588.3 KB</t>
         </is>
       </c>
       <c r="E25" s="10" t="inlineStr">
@@ -1450,7 +1456,7 @@
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="11" t="inlineStr">
         <is>
-          <t>images/cable-stayed-bridge-night-illuminated.jpg</t>
+          <t>images/bridge-architecture-bw-lines.jpg</t>
         </is>
       </c>
       <c r="B26" s="11" t="inlineStr">
@@ -1465,7 +1471,7 @@
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>2763.8 KB</t>
+          <t>1303.2 KB</t>
         </is>
       </c>
       <c r="E26" s="12" t="inlineStr">
@@ -1477,7 +1483,7 @@
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>images/erasmus-bridge-rotterdam-abstract.jpg</t>
+          <t>images/bridge-fog-water-minimalist.jpg</t>
         </is>
       </c>
       <c r="B27" s="9" t="inlineStr">
@@ -1492,7 +1498,7 @@
       </c>
       <c r="D27" s="9" t="inlineStr">
         <is>
-          <t>1987.7 KB</t>
+          <t>1629.4 KB</t>
         </is>
       </c>
       <c r="E27" s="10" t="inlineStr">
@@ -1504,7 +1510,7 @@
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="11" t="inlineStr">
         <is>
-          <t>images/erasmus-bridge-rotterdam-daytime.jpg</t>
+          <t>images/brooklyn-bridge-bw.jpg</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
@@ -1519,7 +1525,7 @@
       </c>
       <c r="D28" s="11" t="inlineStr">
         <is>
-          <t>2735.6 KB</t>
+          <t>4581.0 KB</t>
         </is>
       </c>
       <c r="E28" s="12" t="inlineStr">
@@ -1531,7 +1537,7 @@
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="9" t="inlineStr">
         <is>
-          <t>images/erasmus-bridge-rotterdam-grayscale.jpg</t>
+          <t>images/cable-bridge-dark-sky-dramatic.jpg</t>
         </is>
       </c>
       <c r="B29" s="9" t="inlineStr">
@@ -1546,7 +1552,7 @@
       </c>
       <c r="D29" s="9" t="inlineStr">
         <is>
-          <t>2134.6 KB</t>
+          <t>612.4 KB</t>
         </is>
       </c>
       <c r="E29" s="10" t="inlineStr">
@@ -1558,7 +1564,7 @@
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="11" t="inlineStr">
         <is>
-          <t>images/long-bridge-sunset-dramatic.jpg</t>
+          <t>images/cable-bridge-geometric-perspective.jpg</t>
         </is>
       </c>
       <c r="B30" s="11" t="inlineStr">
@@ -1573,7 +1579,7 @@
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>1619.2 KB</t>
+          <t>1287.9 KB</t>
         </is>
       </c>
       <c r="E30" s="12" t="inlineStr">
@@ -1585,7 +1591,7 @@
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>images/modern-bridge-bw-dramatic.jpg</t>
+          <t>images/cable-bridge-golden-hour.jpg</t>
         </is>
       </c>
       <c r="B31" s="9" t="inlineStr">
@@ -1600,7 +1606,7 @@
       </c>
       <c r="D31" s="9" t="inlineStr">
         <is>
-          <t>1444.4 KB</t>
+          <t>2521.7 KB</t>
         </is>
       </c>
       <c r="E31" s="10" t="inlineStr">
@@ -1612,7 +1618,7 @@
     <row r="32" ht="16" customHeight="1">
       <c r="A32" s="11" t="inlineStr">
         <is>
-          <t>images/modern-cable-bridge-calm-water.jpg</t>
+          <t>images/cable-bridge-grayscale-dramatic.jpg</t>
         </is>
       </c>
       <c r="B32" s="11" t="inlineStr">
@@ -1627,7 +1633,7 @@
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>4010.0 KB</t>
+          <t>1669.8 KB</t>
         </is>
       </c>
       <c r="E32" s="12" t="inlineStr">
@@ -1639,7 +1645,7 @@
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>images/pedestrian-bridge-bw-modern.jpg</t>
+          <t>images/cable-stayed-bridge-night-illuminated.jpg</t>
         </is>
       </c>
       <c r="B33" s="9" t="inlineStr">
@@ -1654,7 +1660,7 @@
       </c>
       <c r="D33" s="9" t="inlineStr">
         <is>
-          <t>5152.5 KB</t>
+          <t>2763.8 KB</t>
         </is>
       </c>
       <c r="E33" s="10" t="inlineStr">
@@ -1666,7 +1672,7 @@
     <row r="34" ht="16" customHeight="1">
       <c r="A34" s="11" t="inlineStr">
         <is>
-          <t>images/rotterdam-bridge-cityscape.jpg</t>
+          <t>images/erasmus-bridge-rotterdam-abstract.jpg</t>
         </is>
       </c>
       <c r="B34" s="11" t="inlineStr">
@@ -1681,7 +1687,7 @@
       </c>
       <c r="D34" s="11" t="inlineStr">
         <is>
-          <t>4795.7 KB</t>
+          <t>1987.7 KB</t>
         </is>
       </c>
       <c r="E34" s="12" t="inlineStr">
@@ -1693,7 +1699,7 @@
     <row r="35" ht="16" customHeight="1">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>images/shutterstock_1510566293_RoyalWelshbrug_zwart_1920x1280px_dark.jpg</t>
+          <t>images/erasmus-bridge-rotterdam-daytime.jpg</t>
         </is>
       </c>
       <c r="B35" s="9" t="inlineStr">
@@ -1708,7 +1714,7 @@
       </c>
       <c r="D35" s="9" t="inlineStr">
         <is>
-          <t>1674.8 KB</t>
+          <t>2735.6 KB</t>
         </is>
       </c>
       <c r="E35" s="10" t="inlineStr">
@@ -1720,7 +1726,7 @@
     <row r="36" ht="16" customHeight="1">
       <c r="A36" s="11" t="inlineStr">
         <is>
-          <t>images/slides/Erasmusbrug_zwart-16x9.jpg</t>
+          <t>images/erasmus-bridge-rotterdam-grayscale.jpg</t>
         </is>
       </c>
       <c r="B36" s="11" t="inlineStr">
@@ -1735,7 +1741,7 @@
       </c>
       <c r="D36" s="11" t="inlineStr">
         <is>
-          <t>405.6 KB</t>
+          <t>2134.6 KB</t>
         </is>
       </c>
       <c r="E36" s="12" t="inlineStr">
@@ -1747,7 +1753,7 @@
     <row r="37" ht="16" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>images/slides/Erasmusbrug_zwart-1x1.jpg</t>
+          <t>images/long-bridge-sunset-dramatic.jpg</t>
         </is>
       </c>
       <c r="B37" s="9" t="inlineStr">
@@ -1762,7 +1768,7 @@
       </c>
       <c r="D37" s="9" t="inlineStr">
         <is>
-          <t>252.9 KB</t>
+          <t>1619.2 KB</t>
         </is>
       </c>
       <c r="E37" s="10" t="inlineStr">
@@ -1774,7 +1780,7 @@
     <row r="38" ht="16" customHeight="1">
       <c r="A38" s="11" t="inlineStr">
         <is>
-          <t>images/slides/Erasmusbrug_zwart-2x1.jpg</t>
+          <t>images/manifest.json</t>
         </is>
       </c>
       <c r="B38" s="11" t="inlineStr">
@@ -1784,12 +1790,12 @@
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>JPEG</t>
+          <t>JSON</t>
         </is>
       </c>
       <c r="D38" s="11" t="inlineStr">
         <is>
-          <t>372.8 KB</t>
+          <t>17.2 KB</t>
         </is>
       </c>
       <c r="E38" s="12" t="inlineStr">
@@ -1801,7 +1807,7 @@
     <row r="39" ht="16" customHeight="1">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>images/slides/Nesciobrug-16x9.jpg</t>
+          <t>images/modern-bridge-bw-dramatic.jpg</t>
         </is>
       </c>
       <c r="B39" s="9" t="inlineStr">
@@ -1816,7 +1822,7 @@
       </c>
       <c r="D39" s="9" t="inlineStr">
         <is>
-          <t>370.9 KB</t>
+          <t>1444.4 KB</t>
         </is>
       </c>
       <c r="E39" s="10" t="inlineStr">
@@ -1828,7 +1834,7 @@
     <row r="40" ht="16" customHeight="1">
       <c r="A40" s="11" t="inlineStr">
         <is>
-          <t>images/slides/Nesciobrug-1x1.jpg</t>
+          <t>images/modern-cable-bridge-calm-water.jpg</t>
         </is>
       </c>
       <c r="B40" s="11" t="inlineStr">
@@ -1843,7 +1849,7 @@
       </c>
       <c r="D40" s="11" t="inlineStr">
         <is>
-          <t>254.1 KB</t>
+          <t>4010.0 KB</t>
         </is>
       </c>
       <c r="E40" s="12" t="inlineStr">
@@ -1855,7 +1861,7 @@
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>images/slides/Nesciobrug-2x1.jpg</t>
+          <t>images/pedestrian-bridge-bw-modern.jpg</t>
         </is>
       </c>
       <c r="B41" s="9" t="inlineStr">
@@ -1870,7 +1876,7 @@
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>318.8 KB</t>
+          <t>5152.5 KB</t>
         </is>
       </c>
       <c r="E41" s="10" t="inlineStr">
@@ -1882,7 +1888,7 @@
     <row r="42" ht="16" customHeight="1">
       <c r="A42" s="11" t="inlineStr">
         <is>
-          <t>images/slides/Pythonbrug_Amsterdam_contrast-16x9.jpg</t>
+          <t>images/rotterdam-bridge-cityscape.jpg</t>
         </is>
       </c>
       <c r="B42" s="11" t="inlineStr">
@@ -1897,7 +1903,7 @@
       </c>
       <c r="D42" s="11" t="inlineStr">
         <is>
-          <t>309.0 KB</t>
+          <t>4795.7 KB</t>
         </is>
       </c>
       <c r="E42" s="12" t="inlineStr">
@@ -1909,7 +1915,7 @@
     <row r="43" ht="16" customHeight="1">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>images/slides/Pythonbrug_Amsterdam_contrast-1x1.jpg</t>
+          <t>images/shutterstock_1510566293_RoyalWelshbrug_zwart_1920x1280px_dark.jpg</t>
         </is>
       </c>
       <c r="B43" s="9" t="inlineStr">
@@ -1924,7 +1930,7 @@
       </c>
       <c r="D43" s="9" t="inlineStr">
         <is>
-          <t>185.3 KB</t>
+          <t>1674.8 KB</t>
         </is>
       </c>
       <c r="E43" s="10" t="inlineStr">
@@ -1936,7 +1942,7 @@
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="11" t="inlineStr">
         <is>
-          <t>images/slides/Pythonbrug_Amsterdam_contrast-2x1.jpg</t>
+          <t>images/slides/Erasmusbrug_zwart-16x9.jpg</t>
         </is>
       </c>
       <c r="B44" s="11" t="inlineStr">
@@ -1951,7 +1957,7 @@
       </c>
       <c r="D44" s="11" t="inlineStr">
         <is>
-          <t>292.1 KB</t>
+          <t>405.6 KB</t>
         </is>
       </c>
       <c r="E44" s="12" t="inlineStr">
@@ -1963,7 +1969,7 @@
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>images/slides/bridge-architecture-bw-lines-16x9.jpg</t>
+          <t>images/slides/Erasmusbrug_zwart-1x1.jpg</t>
         </is>
       </c>
       <c r="B45" s="9" t="inlineStr">
@@ -1978,7 +1984,7 @@
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>584.4 KB</t>
+          <t>252.9 KB</t>
         </is>
       </c>
       <c r="E45" s="10" t="inlineStr">
@@ -1990,7 +1996,7 @@
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="11" t="inlineStr">
         <is>
-          <t>images/slides/bridge-architecture-bw-lines-1x1.jpg</t>
+          <t>images/slides/Erasmusbrug_zwart-2x1.jpg</t>
         </is>
       </c>
       <c r="B46" s="11" t="inlineStr">
@@ -2005,7 +2011,7 @@
       </c>
       <c r="D46" s="11" t="inlineStr">
         <is>
-          <t>333.4 KB</t>
+          <t>372.8 KB</t>
         </is>
       </c>
       <c r="E46" s="12" t="inlineStr">
@@ -2017,7 +2023,7 @@
     <row r="47" ht="16" customHeight="1">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>images/slides/bridge-architecture-bw-lines-2x1.jpg</t>
+          <t>images/slides/Nesciobrug-16x9.jpg</t>
         </is>
       </c>
       <c r="B47" s="9" t="inlineStr">
@@ -2032,7 +2038,7 @@
       </c>
       <c r="D47" s="9" t="inlineStr">
         <is>
-          <t>536.5 KB</t>
+          <t>370.9 KB</t>
         </is>
       </c>
       <c r="E47" s="10" t="inlineStr">
@@ -2044,7 +2050,7 @@
     <row r="48" ht="16" customHeight="1">
       <c r="A48" s="11" t="inlineStr">
         <is>
-          <t>images/slides/bridge-fog-water-minimalist-16x9.jpg</t>
+          <t>images/slides/Nesciobrug-1x1.jpg</t>
         </is>
       </c>
       <c r="B48" s="11" t="inlineStr">
@@ -2059,7 +2065,7 @@
       </c>
       <c r="D48" s="11" t="inlineStr">
         <is>
-          <t>358.9 KB</t>
+          <t>254.1 KB</t>
         </is>
       </c>
       <c r="E48" s="12" t="inlineStr">
@@ -2071,7 +2077,7 @@
     <row r="49" ht="16" customHeight="1">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>images/slides/bridge-fog-water-minimalist-1x1.jpg</t>
+          <t>images/slides/Nesciobrug-2x1.jpg</t>
         </is>
       </c>
       <c r="B49" s="9" t="inlineStr">
@@ -2086,7 +2092,7 @@
       </c>
       <c r="D49" s="9" t="inlineStr">
         <is>
-          <t>130.7 KB</t>
+          <t>318.8 KB</t>
         </is>
       </c>
       <c r="E49" s="10" t="inlineStr">
@@ -2098,7 +2104,7 @@
     <row r="50" ht="16" customHeight="1">
       <c r="A50" s="11" t="inlineStr">
         <is>
-          <t>images/slides/bridge-fog-water-minimalist-2x1.jpg</t>
+          <t>images/slides/Pythonbrug_Amsterdam_contrast-16x9.jpg</t>
         </is>
       </c>
       <c r="B50" s="11" t="inlineStr">
@@ -2113,7 +2119,7 @@
       </c>
       <c r="D50" s="11" t="inlineStr">
         <is>
-          <t>323.4 KB</t>
+          <t>309.0 KB</t>
         </is>
       </c>
       <c r="E50" s="12" t="inlineStr">
@@ -2125,7 +2131,7 @@
     <row r="51" ht="16" customHeight="1">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>images/slides/brooklyn-bridge-bw-16x9.jpg</t>
+          <t>images/slides/Pythonbrug_Amsterdam_contrast-1x1.jpg</t>
         </is>
       </c>
       <c r="B51" s="9" t="inlineStr">
@@ -2140,7 +2146,7 @@
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>583.8 KB</t>
+          <t>185.3 KB</t>
         </is>
       </c>
       <c r="E51" s="10" t="inlineStr">
@@ -2152,7 +2158,7 @@
     <row r="52" ht="16" customHeight="1">
       <c r="A52" s="11" t="inlineStr">
         <is>
-          <t>images/slides/brooklyn-bridge-bw-1x1.jpg</t>
+          <t>images/slides/Pythonbrug_Amsterdam_contrast-2x1.jpg</t>
         </is>
       </c>
       <c r="B52" s="11" t="inlineStr">
@@ -2167,7 +2173,7 @@
       </c>
       <c r="D52" s="11" t="inlineStr">
         <is>
-          <t>340.2 KB</t>
+          <t>292.1 KB</t>
         </is>
       </c>
       <c r="E52" s="12" t="inlineStr">
@@ -2179,7 +2185,7 @@
     <row r="53" ht="16" customHeight="1">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>images/slides/brooklyn-bridge-bw-2x1.jpg</t>
+          <t>images/slides/bridge-architecture-bw-lines-16x9.jpg</t>
         </is>
       </c>
       <c r="B53" s="9" t="inlineStr">
@@ -2194,7 +2200,7 @@
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>516.4 KB</t>
+          <t>584.4 KB</t>
         </is>
       </c>
       <c r="E53" s="10" t="inlineStr">
@@ -2206,7 +2212,7 @@
     <row r="54" ht="16" customHeight="1">
       <c r="A54" s="11" t="inlineStr">
         <is>
-          <t>images/slides/cable-bridge-dark-sky-dramatic-16x9.jpg</t>
+          <t>images/slides/bridge-architecture-bw-lines-1x1.jpg</t>
         </is>
       </c>
       <c r="B54" s="11" t="inlineStr">
@@ -2221,7 +2227,7 @@
       </c>
       <c r="D54" s="11" t="inlineStr">
         <is>
-          <t>214.3 KB</t>
+          <t>333.4 KB</t>
         </is>
       </c>
       <c r="E54" s="12" t="inlineStr">
@@ -2233,7 +2239,7 @@
     <row r="55" ht="16" customHeight="1">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>images/slides/cable-bridge-dark-sky-dramatic-1x1.jpg</t>
+          <t>images/slides/bridge-architecture-bw-lines-2x1.jpg</t>
         </is>
       </c>
       <c r="B55" s="9" t="inlineStr">
@@ -2248,7 +2254,7 @@
       </c>
       <c r="D55" s="9" t="inlineStr">
         <is>
-          <t>148.8 KB</t>
+          <t>536.5 KB</t>
         </is>
       </c>
       <c r="E55" s="10" t="inlineStr">
@@ -2260,7 +2266,7 @@
     <row r="56" ht="16" customHeight="1">
       <c r="A56" s="11" t="inlineStr">
         <is>
-          <t>images/slides/cable-bridge-dark-sky-dramatic-2x1.jpg</t>
+          <t>images/slides/bridge-fog-water-minimalist-16x9.jpg</t>
         </is>
       </c>
       <c r="B56" s="11" t="inlineStr">
@@ -2275,7 +2281,7 @@
       </c>
       <c r="D56" s="11" t="inlineStr">
         <is>
-          <t>196.7 KB</t>
+          <t>358.9 KB</t>
         </is>
       </c>
       <c r="E56" s="12" t="inlineStr">
@@ -2287,7 +2293,7 @@
     <row r="57" ht="16" customHeight="1">
       <c r="A57" s="9" t="inlineStr">
         <is>
-          <t>images/slides/cable-bridge-geometric-perspective-16x9.jpg</t>
+          <t>images/slides/bridge-fog-water-minimalist-1x1.jpg</t>
         </is>
       </c>
       <c r="B57" s="9" t="inlineStr">
@@ -2302,7 +2308,7 @@
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>266.6 KB</t>
+          <t>130.7 KB</t>
         </is>
       </c>
       <c r="E57" s="10" t="inlineStr">
@@ -2314,7 +2320,7 @@
     <row r="58" ht="16" customHeight="1">
       <c r="A58" s="11" t="inlineStr">
         <is>
-          <t>images/slides/cable-bridge-geometric-perspective-1x1.jpg</t>
+          <t>images/slides/bridge-fog-water-minimalist-2x1.jpg</t>
         </is>
       </c>
       <c r="B58" s="11" t="inlineStr">
@@ -2329,7 +2335,7 @@
       </c>
       <c r="D58" s="11" t="inlineStr">
         <is>
-          <t>161.0 KB</t>
+          <t>323.4 KB</t>
         </is>
       </c>
       <c r="E58" s="12" t="inlineStr">
@@ -2341,7 +2347,7 @@
     <row r="59" ht="16" customHeight="1">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>images/slides/cable-bridge-geometric-perspective-2x1.jpg</t>
+          <t>images/slides/brooklyn-bridge-bw-16x9.jpg</t>
         </is>
       </c>
       <c r="B59" s="9" t="inlineStr">
@@ -2356,7 +2362,7 @@
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>234.2 KB</t>
+          <t>583.8 KB</t>
         </is>
       </c>
       <c r="E59" s="10" t="inlineStr">
@@ -2368,7 +2374,7 @@
     <row r="60" ht="16" customHeight="1">
       <c r="A60" s="11" t="inlineStr">
         <is>
-          <t>images/slides/cable-bridge-golden-hour-16x9.jpg</t>
+          <t>images/slides/brooklyn-bridge-bw-1x1.jpg</t>
         </is>
       </c>
       <c r="B60" s="11" t="inlineStr">
@@ -2383,7 +2389,7 @@
       </c>
       <c r="D60" s="11" t="inlineStr">
         <is>
-          <t>698.7 KB</t>
+          <t>340.2 KB</t>
         </is>
       </c>
       <c r="E60" s="12" t="inlineStr">
@@ -2395,7 +2401,7 @@
     <row r="61" ht="16" customHeight="1">
       <c r="A61" s="9" t="inlineStr">
         <is>
-          <t>images/slides/cable-bridge-golden-hour-1x1.jpg</t>
+          <t>images/slides/brooklyn-bridge-bw-2x1.jpg</t>
         </is>
       </c>
       <c r="B61" s="9" t="inlineStr">
@@ -2410,7 +2416,7 @@
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>380.4 KB</t>
+          <t>516.4 KB</t>
         </is>
       </c>
       <c r="E61" s="10" t="inlineStr">
@@ -2422,7 +2428,7 @@
     <row r="62" ht="16" customHeight="1">
       <c r="A62" s="11" t="inlineStr">
         <is>
-          <t>images/slides/cable-bridge-golden-hour-2x1.jpg</t>
+          <t>images/slides/cable-bridge-dark-sky-dramatic-16x9.jpg</t>
         </is>
       </c>
       <c r="B62" s="11" t="inlineStr">
@@ -2437,7 +2443,7 @@
       </c>
       <c r="D62" s="11" t="inlineStr">
         <is>
-          <t>622.6 KB</t>
+          <t>214.3 KB</t>
         </is>
       </c>
       <c r="E62" s="12" t="inlineStr">
@@ -2449,7 +2455,7 @@
     <row r="63" ht="16" customHeight="1">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t>images/slides/cable-bridge-grayscale-dramatic-16x9.jpg</t>
+          <t>images/slides/cable-bridge-dark-sky-dramatic-1x1.jpg</t>
         </is>
       </c>
       <c r="B63" s="9" t="inlineStr">
@@ -2464,7 +2470,7 @@
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>195.7 KB</t>
+          <t>148.8 KB</t>
         </is>
       </c>
       <c r="E63" s="10" t="inlineStr">
@@ -2476,7 +2482,7 @@
     <row r="64" ht="16" customHeight="1">
       <c r="A64" s="11" t="inlineStr">
         <is>
-          <t>images/slides/cable-bridge-grayscale-dramatic-1x1.jpg</t>
+          <t>images/slides/cable-bridge-dark-sky-dramatic-2x1.jpg</t>
         </is>
       </c>
       <c r="B64" s="11" t="inlineStr">
@@ -2491,7 +2497,7 @@
       </c>
       <c r="D64" s="11" t="inlineStr">
         <is>
-          <t>117.1 KB</t>
+          <t>196.7 KB</t>
         </is>
       </c>
       <c r="E64" s="12" t="inlineStr">
@@ -2503,7 +2509,7 @@
     <row r="65" ht="16" customHeight="1">
       <c r="A65" s="9" t="inlineStr">
         <is>
-          <t>images/slides/cable-bridge-grayscale-dramatic-2x1.jpg</t>
+          <t>images/slides/cable-bridge-geometric-perspective-16x9.jpg</t>
         </is>
       </c>
       <c r="B65" s="9" t="inlineStr">
@@ -2518,7 +2524,7 @@
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>176.5 KB</t>
+          <t>266.6 KB</t>
         </is>
       </c>
       <c r="E65" s="10" t="inlineStr">
@@ -2530,7 +2536,7 @@
     <row r="66" ht="16" customHeight="1">
       <c r="A66" s="11" t="inlineStr">
         <is>
-          <t>images/slides/cable-stayed-bridge-night-illuminated-16x9.jpg</t>
+          <t>images/slides/cable-bridge-geometric-perspective-1x1.jpg</t>
         </is>
       </c>
       <c r="B66" s="11" t="inlineStr">
@@ -2545,7 +2551,7 @@
       </c>
       <c r="D66" s="11" t="inlineStr">
         <is>
-          <t>436.4 KB</t>
+          <t>161.0 KB</t>
         </is>
       </c>
       <c r="E66" s="12" t="inlineStr">
@@ -2557,7 +2563,7 @@
     <row r="67" ht="16" customHeight="1">
       <c r="A67" s="9" t="inlineStr">
         <is>
-          <t>images/slides/cable-stayed-bridge-night-illuminated-1x1.jpg</t>
+          <t>images/slides/cable-bridge-geometric-perspective-2x1.jpg</t>
         </is>
       </c>
       <c r="B67" s="9" t="inlineStr">
@@ -2572,7 +2578,7 @@
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>263.0 KB</t>
+          <t>234.2 KB</t>
         </is>
       </c>
       <c r="E67" s="10" t="inlineStr">
@@ -2584,7 +2590,7 @@
     <row r="68" ht="16" customHeight="1">
       <c r="A68" s="11" t="inlineStr">
         <is>
-          <t>images/slides/cable-stayed-bridge-night-illuminated-2x1.jpg</t>
+          <t>images/slides/cable-bridge-golden-hour-16x9.jpg</t>
         </is>
       </c>
       <c r="B68" s="11" t="inlineStr">
@@ -2599,7 +2605,7 @@
       </c>
       <c r="D68" s="11" t="inlineStr">
         <is>
-          <t>422.6 KB</t>
+          <t>698.7 KB</t>
         </is>
       </c>
       <c r="E68" s="12" t="inlineStr">
@@ -2611,7 +2617,7 @@
     <row r="69" ht="16" customHeight="1">
       <c r="A69" s="9" t="inlineStr">
         <is>
-          <t>images/slides/erasmus-bridge-rotterdam-abstract-16x9.jpg</t>
+          <t>images/slides/cable-bridge-golden-hour-1x1.jpg</t>
         </is>
       </c>
       <c r="B69" s="9" t="inlineStr">
@@ -2626,7 +2632,7 @@
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>303.3 KB</t>
+          <t>380.4 KB</t>
         </is>
       </c>
       <c r="E69" s="10" t="inlineStr">
@@ -2638,7 +2644,7 @@
     <row r="70" ht="16" customHeight="1">
       <c r="A70" s="11" t="inlineStr">
         <is>
-          <t>images/slides/erasmus-bridge-rotterdam-abstract-1x1.jpg</t>
+          <t>images/slides/cable-bridge-golden-hour-2x1.jpg</t>
         </is>
       </c>
       <c r="B70" s="11" t="inlineStr">
@@ -2653,7 +2659,7 @@
       </c>
       <c r="D70" s="11" t="inlineStr">
         <is>
-          <t>190.3 KB</t>
+          <t>622.6 KB</t>
         </is>
       </c>
       <c r="E70" s="12" t="inlineStr">
@@ -2665,7 +2671,7 @@
     <row r="71" ht="16" customHeight="1">
       <c r="A71" s="9" t="inlineStr">
         <is>
-          <t>images/slides/erasmus-bridge-rotterdam-abstract-2x1.jpg</t>
+          <t>images/slides/cable-bridge-grayscale-dramatic-16x9.jpg</t>
         </is>
       </c>
       <c r="B71" s="9" t="inlineStr">
@@ -2680,7 +2686,7 @@
       </c>
       <c r="D71" s="9" t="inlineStr">
         <is>
-          <t>274.6 KB</t>
+          <t>195.7 KB</t>
         </is>
       </c>
       <c r="E71" s="10" t="inlineStr">
@@ -2692,7 +2698,7 @@
     <row r="72" ht="16" customHeight="1">
       <c r="A72" s="11" t="inlineStr">
         <is>
-          <t>images/slides/erasmus-bridge-rotterdam-daytime-16x9.jpg</t>
+          <t>images/slides/cable-bridge-grayscale-dramatic-1x1.jpg</t>
         </is>
       </c>
       <c r="B72" s="11" t="inlineStr">
@@ -2707,7 +2713,7 @@
       </c>
       <c r="D72" s="11" t="inlineStr">
         <is>
-          <t>534.4 KB</t>
+          <t>117.1 KB</t>
         </is>
       </c>
       <c r="E72" s="12" t="inlineStr">
@@ -2719,7 +2725,7 @@
     <row r="73" ht="16" customHeight="1">
       <c r="A73" s="9" t="inlineStr">
         <is>
-          <t>images/slides/erasmus-bridge-rotterdam-daytime-1x1.jpg</t>
+          <t>images/slides/cable-bridge-grayscale-dramatic-2x1.jpg</t>
         </is>
       </c>
       <c r="B73" s="9" t="inlineStr">
@@ -2734,7 +2740,7 @@
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>306.7 KB</t>
+          <t>176.5 KB</t>
         </is>
       </c>
       <c r="E73" s="10" t="inlineStr">
@@ -2746,7 +2752,7 @@
     <row r="74" ht="16" customHeight="1">
       <c r="A74" s="11" t="inlineStr">
         <is>
-          <t>images/slides/erasmus-bridge-rotterdam-daytime-2x1.jpg</t>
+          <t>images/slides/cable-stayed-bridge-night-illuminated-16x9.jpg</t>
         </is>
       </c>
       <c r="B74" s="11" t="inlineStr">
@@ -2761,7 +2767,7 @@
       </c>
       <c r="D74" s="11" t="inlineStr">
         <is>
-          <t>471.3 KB</t>
+          <t>436.4 KB</t>
         </is>
       </c>
       <c r="E74" s="12" t="inlineStr">
@@ -2773,7 +2779,7 @@
     <row r="75" ht="16" customHeight="1">
       <c r="A75" s="9" t="inlineStr">
         <is>
-          <t>images/slides/erasmus-bridge-rotterdam-grayscale-16x9.jpg</t>
+          <t>images/slides/cable-stayed-bridge-night-illuminated-1x1.jpg</t>
         </is>
       </c>
       <c r="B75" s="9" t="inlineStr">
@@ -2788,7 +2794,7 @@
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>287.1 KB</t>
+          <t>263.0 KB</t>
         </is>
       </c>
       <c r="E75" s="10" t="inlineStr">
@@ -2800,7 +2806,7 @@
     <row r="76" ht="16" customHeight="1">
       <c r="A76" s="11" t="inlineStr">
         <is>
-          <t>images/slides/erasmus-bridge-rotterdam-grayscale-1x1.jpg</t>
+          <t>images/slides/cable-stayed-bridge-night-illuminated-2x1.jpg</t>
         </is>
       </c>
       <c r="B76" s="11" t="inlineStr">
@@ -2815,7 +2821,7 @@
       </c>
       <c r="D76" s="11" t="inlineStr">
         <is>
-          <t>156.5 KB</t>
+          <t>422.6 KB</t>
         </is>
       </c>
       <c r="E76" s="12" t="inlineStr">
@@ -2827,7 +2833,7 @@
     <row r="77" ht="16" customHeight="1">
       <c r="A77" s="9" t="inlineStr">
         <is>
-          <t>images/slides/erasmus-bridge-rotterdam-grayscale-2x1.jpg</t>
+          <t>images/slides/erasmus-bridge-rotterdam-abstract-16x9.jpg</t>
         </is>
       </c>
       <c r="B77" s="9" t="inlineStr">
@@ -2842,7 +2848,7 @@
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>269.8 KB</t>
+          <t>303.3 KB</t>
         </is>
       </c>
       <c r="E77" s="10" t="inlineStr">
@@ -2854,7 +2860,7 @@
     <row r="78" ht="16" customHeight="1">
       <c r="A78" s="11" t="inlineStr">
         <is>
-          <t>images/slides/long-bridge-sunset-dramatic-16x9.jpg</t>
+          <t>images/slides/erasmus-bridge-rotterdam-abstract-1x1.jpg</t>
         </is>
       </c>
       <c r="B78" s="11" t="inlineStr">
@@ -2869,7 +2875,7 @@
       </c>
       <c r="D78" s="11" t="inlineStr">
         <is>
-          <t>416.9 KB</t>
+          <t>190.3 KB</t>
         </is>
       </c>
       <c r="E78" s="12" t="inlineStr">
@@ -2881,7 +2887,7 @@
     <row r="79" ht="16" customHeight="1">
       <c r="A79" s="9" t="inlineStr">
         <is>
-          <t>images/slides/long-bridge-sunset-dramatic-1x1.jpg</t>
+          <t>images/slides/erasmus-bridge-rotterdam-abstract-2x1.jpg</t>
         </is>
       </c>
       <c r="B79" s="9" t="inlineStr">
@@ -2896,7 +2902,7 @@
       </c>
       <c r="D79" s="9" t="inlineStr">
         <is>
-          <t>270.0 KB</t>
+          <t>274.6 KB</t>
         </is>
       </c>
       <c r="E79" s="10" t="inlineStr">
@@ -2908,7 +2914,7 @@
     <row r="80" ht="16" customHeight="1">
       <c r="A80" s="11" t="inlineStr">
         <is>
-          <t>images/slides/long-bridge-sunset-dramatic-2x1.jpg</t>
+          <t>images/slides/erasmus-bridge-rotterdam-daytime-16x9.jpg</t>
         </is>
       </c>
       <c r="B80" s="11" t="inlineStr">
@@ -2923,7 +2929,7 @@
       </c>
       <c r="D80" s="11" t="inlineStr">
         <is>
-          <t>382.5 KB</t>
+          <t>534.4 KB</t>
         </is>
       </c>
       <c r="E80" s="12" t="inlineStr">
@@ -2935,7 +2941,7 @@
     <row r="81" ht="16" customHeight="1">
       <c r="A81" s="9" t="inlineStr">
         <is>
-          <t>images/slides/modern-bridge-bw-dramatic-16x9.jpg</t>
+          <t>images/slides/erasmus-bridge-rotterdam-daytime-1x1.jpg</t>
         </is>
       </c>
       <c r="B81" s="9" t="inlineStr">
@@ -2950,7 +2956,7 @@
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>218.2 KB</t>
+          <t>306.7 KB</t>
         </is>
       </c>
       <c r="E81" s="10" t="inlineStr">
@@ -2962,7 +2968,7 @@
     <row r="82" ht="16" customHeight="1">
       <c r="A82" s="11" t="inlineStr">
         <is>
-          <t>images/slides/modern-bridge-bw-dramatic-1x1.jpg</t>
+          <t>images/slides/erasmus-bridge-rotterdam-daytime-2x1.jpg</t>
         </is>
       </c>
       <c r="B82" s="11" t="inlineStr">
@@ -2977,7 +2983,7 @@
       </c>
       <c r="D82" s="11" t="inlineStr">
         <is>
-          <t>140.8 KB</t>
+          <t>471.3 KB</t>
         </is>
       </c>
       <c r="E82" s="12" t="inlineStr">
@@ -2989,7 +2995,7 @@
     <row r="83" ht="16" customHeight="1">
       <c r="A83" s="9" t="inlineStr">
         <is>
-          <t>images/slides/modern-bridge-bw-dramatic-2x1.jpg</t>
+          <t>images/slides/erasmus-bridge-rotterdam-grayscale-16x9.jpg</t>
         </is>
       </c>
       <c r="B83" s="9" t="inlineStr">
@@ -3004,7 +3010,7 @@
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>198.6 KB</t>
+          <t>287.1 KB</t>
         </is>
       </c>
       <c r="E83" s="10" t="inlineStr">
@@ -3016,7 +3022,7 @@
     <row r="84" ht="16" customHeight="1">
       <c r="A84" s="11" t="inlineStr">
         <is>
-          <t>images/slides/modern-cable-bridge-calm-water-16x9.jpg</t>
+          <t>images/slides/erasmus-bridge-rotterdam-grayscale-1x1.jpg</t>
         </is>
       </c>
       <c r="B84" s="11" t="inlineStr">
@@ -3031,7 +3037,7 @@
       </c>
       <c r="D84" s="11" t="inlineStr">
         <is>
-          <t>269.2 KB</t>
+          <t>156.5 KB</t>
         </is>
       </c>
       <c r="E84" s="12" t="inlineStr">
@@ -3043,7 +3049,7 @@
     <row r="85" ht="16" customHeight="1">
       <c r="A85" s="9" t="inlineStr">
         <is>
-          <t>images/slides/modern-cable-bridge-calm-water-1x1.jpg</t>
+          <t>images/slides/erasmus-bridge-rotterdam-grayscale-2x1.jpg</t>
         </is>
       </c>
       <c r="B85" s="9" t="inlineStr">
@@ -3058,7 +3064,7 @@
       </c>
       <c r="D85" s="9" t="inlineStr">
         <is>
-          <t>151.3 KB</t>
+          <t>269.8 KB</t>
         </is>
       </c>
       <c r="E85" s="10" t="inlineStr">
@@ -3070,7 +3076,7 @@
     <row r="86" ht="16" customHeight="1">
       <c r="A86" s="11" t="inlineStr">
         <is>
-          <t>images/slides/modern-cable-bridge-calm-water-2x1.jpg</t>
+          <t>images/slides/long-bridge-sunset-dramatic-16x9.jpg</t>
         </is>
       </c>
       <c r="B86" s="11" t="inlineStr">
@@ -3085,7 +3091,7 @@
       </c>
       <c r="D86" s="11" t="inlineStr">
         <is>
-          <t>254.5 KB</t>
+          <t>416.9 KB</t>
         </is>
       </c>
       <c r="E86" s="12" t="inlineStr">
@@ -3097,7 +3103,7 @@
     <row r="87" ht="16" customHeight="1">
       <c r="A87" s="9" t="inlineStr">
         <is>
-          <t>images/slides/pedestrian-bridge-bw-modern-16x9.jpg</t>
+          <t>images/slides/long-bridge-sunset-dramatic-1x1.jpg</t>
         </is>
       </c>
       <c r="B87" s="9" t="inlineStr">
@@ -3112,7 +3118,7 @@
       </c>
       <c r="D87" s="9" t="inlineStr">
         <is>
-          <t>548.7 KB</t>
+          <t>270.0 KB</t>
         </is>
       </c>
       <c r="E87" s="10" t="inlineStr">
@@ -3124,7 +3130,7 @@
     <row r="88" ht="16" customHeight="1">
       <c r="A88" s="11" t="inlineStr">
         <is>
-          <t>images/slides/pedestrian-bridge-bw-modern-1x1.jpg</t>
+          <t>images/slides/long-bridge-sunset-dramatic-2x1.jpg</t>
         </is>
       </c>
       <c r="B88" s="11" t="inlineStr">
@@ -3139,7 +3145,7 @@
       </c>
       <c r="D88" s="11" t="inlineStr">
         <is>
-          <t>297.4 KB</t>
+          <t>382.5 KB</t>
         </is>
       </c>
       <c r="E88" s="12" t="inlineStr">
@@ -3151,7 +3157,7 @@
     <row r="89" ht="16" customHeight="1">
       <c r="A89" s="9" t="inlineStr">
         <is>
-          <t>images/slides/pedestrian-bridge-bw-modern-2x1.jpg</t>
+          <t>images/slides/modern-bridge-bw-dramatic-16x9.jpg</t>
         </is>
       </c>
       <c r="B89" s="9" t="inlineStr">
@@ -3166,7 +3172,7 @@
       </c>
       <c r="D89" s="9" t="inlineStr">
         <is>
-          <t>496.6 KB</t>
+          <t>218.2 KB</t>
         </is>
       </c>
       <c r="E89" s="10" t="inlineStr">
@@ -3178,7 +3184,7 @@
     <row r="90" ht="16" customHeight="1">
       <c r="A90" s="11" t="inlineStr">
         <is>
-          <t>images/slides/rotterdam-bridge-cityscape-16x9.jpg</t>
+          <t>images/slides/modern-bridge-bw-dramatic-1x1.jpg</t>
         </is>
       </c>
       <c r="B90" s="11" t="inlineStr">
@@ -3193,7 +3199,7 @@
       </c>
       <c r="D90" s="11" t="inlineStr">
         <is>
-          <t>655.5 KB</t>
+          <t>140.8 KB</t>
         </is>
       </c>
       <c r="E90" s="12" t="inlineStr">
@@ -3205,7 +3211,7 @@
     <row r="91" ht="16" customHeight="1">
       <c r="A91" s="9" t="inlineStr">
         <is>
-          <t>images/slides/rotterdam-bridge-cityscape-1x1.jpg</t>
+          <t>images/slides/modern-bridge-bw-dramatic-2x1.jpg</t>
         </is>
       </c>
       <c r="B91" s="9" t="inlineStr">
@@ -3220,7 +3226,7 @@
       </c>
       <c r="D91" s="9" t="inlineStr">
         <is>
-          <t>343.1 KB</t>
+          <t>198.6 KB</t>
         </is>
       </c>
       <c r="E91" s="10" t="inlineStr">
@@ -3232,7 +3238,7 @@
     <row r="92" ht="16" customHeight="1">
       <c r="A92" s="11" t="inlineStr">
         <is>
-          <t>images/slides/rotterdam-bridge-cityscape-2x1.jpg</t>
+          <t>images/slides/modern-cable-bridge-calm-water-16x9.jpg</t>
         </is>
       </c>
       <c r="B92" s="11" t="inlineStr">
@@ -3247,7 +3253,7 @@
       </c>
       <c r="D92" s="11" t="inlineStr">
         <is>
-          <t>607.0 KB</t>
+          <t>269.2 KB</t>
         </is>
       </c>
       <c r="E92" s="12" t="inlineStr">
@@ -3259,7 +3265,7 @@
     <row r="93" ht="16" customHeight="1">
       <c r="A93" s="9" t="inlineStr">
         <is>
-          <t>images/slides/shutterstock_1510566293_RoyalWelshbrug_zwart_1920x1280px_dark-16x9.jpg</t>
+          <t>images/slides/modern-cable-bridge-calm-water-1x1.jpg</t>
         </is>
       </c>
       <c r="B93" s="9" t="inlineStr">
@@ -3274,7 +3280,7 @@
       </c>
       <c r="D93" s="9" t="inlineStr">
         <is>
-          <t>722.7 KB</t>
+          <t>151.3 KB</t>
         </is>
       </c>
       <c r="E93" s="10" t="inlineStr">
@@ -3286,7 +3292,7 @@
     <row r="94" ht="16" customHeight="1">
       <c r="A94" s="11" t="inlineStr">
         <is>
-          <t>images/slides/shutterstock_1510566293_RoyalWelshbrug_zwart_1920x1280px_dark-1x1.jpg</t>
+          <t>images/slides/modern-cable-bridge-calm-water-2x1.jpg</t>
         </is>
       </c>
       <c r="B94" s="11" t="inlineStr">
@@ -3301,7 +3307,7 @@
       </c>
       <c r="D94" s="11" t="inlineStr">
         <is>
-          <t>418.9 KB</t>
+          <t>254.5 KB</t>
         </is>
       </c>
       <c r="E94" s="12" t="inlineStr">
@@ -3313,7 +3319,7 @@
     <row r="95" ht="16" customHeight="1">
       <c r="A95" s="9" t="inlineStr">
         <is>
-          <t>images/slides/shutterstock_1510566293_RoyalWelshbrug_zwart_1920x1280px_dark-2x1.jpg</t>
+          <t>images/slides/pedestrian-bridge-bw-modern-16x9.jpg</t>
         </is>
       </c>
       <c r="B95" s="9" t="inlineStr">
@@ -3328,7 +3334,7 @@
       </c>
       <c r="D95" s="9" t="inlineStr">
         <is>
-          <t>635.9 KB</t>
+          <t>548.7 KB</t>
         </is>
       </c>
       <c r="E95" s="10" t="inlineStr">
@@ -3340,444 +3346,444 @@
     <row r="96" ht="16" customHeight="1">
       <c r="A96" s="11" t="inlineStr">
         <is>
-          <t>logos/apple-touch-icon-180.png</t>
+          <t>images/slides/pedestrian-bridge-bw-modern-1x1.jpg</t>
         </is>
       </c>
       <c r="B96" s="11" t="inlineStr">
         <is>
-          <t>logos</t>
+          <t>images</t>
         </is>
       </c>
       <c r="C96" s="11" t="inlineStr">
         <is>
-          <t>PNG</t>
+          <t>JPEG</t>
         </is>
       </c>
       <c r="D96" s="11" t="inlineStr">
         <is>
-          <t>18.5 KB</t>
+          <t>297.4 KB</t>
         </is>
       </c>
       <c r="E96" s="12" t="inlineStr">
         <is>
-          <t>Logo asset — apple-touch-icon-180</t>
+          <t>Photography / imagery asset</t>
         </is>
       </c>
     </row>
     <row r="97" ht="16" customHeight="1">
       <c r="A97" s="9" t="inlineStr">
         <is>
-          <t>logos/favicon-192.png</t>
+          <t>images/slides/pedestrian-bridge-bw-modern-2x1.jpg</t>
         </is>
       </c>
       <c r="B97" s="9" t="inlineStr">
         <is>
-          <t>logos</t>
+          <t>images</t>
         </is>
       </c>
       <c r="C97" s="9" t="inlineStr">
         <is>
-          <t>PNG</t>
+          <t>JPEG</t>
         </is>
       </c>
       <c r="D97" s="9" t="inlineStr">
         <is>
-          <t>20.4 KB</t>
+          <t>496.6 KB</t>
         </is>
       </c>
       <c r="E97" s="10" t="inlineStr">
         <is>
-          <t>Logo asset — favicon-192</t>
+          <t>Photography / imagery asset</t>
         </is>
       </c>
     </row>
     <row r="98" ht="16" customHeight="1">
       <c r="A98" s="11" t="inlineStr">
         <is>
-          <t>logos/favicon-32.png</t>
+          <t>images/slides/rotterdam-bridge-cityscape-16x9.jpg</t>
         </is>
       </c>
       <c r="B98" s="11" t="inlineStr">
         <is>
-          <t>logos</t>
+          <t>images</t>
         </is>
       </c>
       <c r="C98" s="11" t="inlineStr">
         <is>
-          <t>PNG</t>
+          <t>JPEG</t>
         </is>
       </c>
       <c r="D98" s="11" t="inlineStr">
         <is>
-          <t>1.1 KB</t>
+          <t>655.5 KB</t>
         </is>
       </c>
       <c r="E98" s="12" t="inlineStr">
         <is>
-          <t>Logo asset — favicon-32</t>
+          <t>Photography / imagery asset</t>
         </is>
       </c>
     </row>
     <row r="99" ht="16" customHeight="1">
       <c r="A99" s="9" t="inlineStr">
         <is>
-          <t>logos/favicon.png</t>
+          <t>images/slides/rotterdam-bridge-cityscape-1x1.jpg</t>
         </is>
       </c>
       <c r="B99" s="9" t="inlineStr">
         <is>
-          <t>logos</t>
+          <t>images</t>
         </is>
       </c>
       <c r="C99" s="9" t="inlineStr">
         <is>
-          <t>PNG</t>
+          <t>JPEG</t>
         </is>
       </c>
       <c r="D99" s="9" t="inlineStr">
         <is>
-          <t>35.2 KB</t>
+          <t>343.1 KB</t>
         </is>
       </c>
       <c r="E99" s="10" t="inlineStr">
         <is>
-          <t>Logo asset — favicon</t>
+          <t>Photography / imagery asset</t>
         </is>
       </c>
     </row>
     <row r="100" ht="16" customHeight="1">
       <c r="A100" s="11" t="inlineStr">
         <is>
-          <t>logos/logo.png</t>
+          <t>images/slides/rotterdam-bridge-cityscape-2x1.jpg</t>
         </is>
       </c>
       <c r="B100" s="11" t="inlineStr">
         <is>
-          <t>logos</t>
+          <t>images</t>
         </is>
       </c>
       <c r="C100" s="11" t="inlineStr">
         <is>
-          <t>PNG</t>
+          <t>JPEG</t>
         </is>
       </c>
       <c r="D100" s="11" t="inlineStr">
         <is>
-          <t>23.2 KB</t>
+          <t>607.0 KB</t>
         </is>
       </c>
       <c r="E100" s="12" t="inlineStr">
         <is>
-          <t>Logo asset — logo</t>
+          <t>Photography / imagery asset</t>
         </is>
       </c>
     </row>
     <row r="101" ht="16" customHeight="1">
       <c r="A101" s="9" t="inlineStr">
         <is>
-          <t>logos/logo.svg</t>
+          <t>images/slides/shutterstock_1510566293_RoyalWelshbrug_zwart_1920x1280px_dark-16x9.jpg</t>
         </is>
       </c>
       <c r="B101" s="9" t="inlineStr">
         <is>
-          <t>logos</t>
+          <t>images</t>
         </is>
       </c>
       <c r="C101" s="9" t="inlineStr">
         <is>
-          <t>SVG</t>
+          <t>JPEG</t>
         </is>
       </c>
       <c r="D101" s="9" t="inlineStr">
         <is>
-          <t>23.7 KB</t>
+          <t>722.7 KB</t>
         </is>
       </c>
       <c r="E101" s="10" t="inlineStr">
         <is>
-          <t>Logo asset — logo</t>
+          <t>Photography / imagery asset</t>
         </is>
       </c>
     </row>
     <row r="102" ht="16" customHeight="1">
       <c r="A102" s="11" t="inlineStr">
         <is>
-          <t>logos/logo_grey.svg</t>
+          <t>images/slides/shutterstock_1510566293_RoyalWelshbrug_zwart_1920x1280px_dark-1x1.jpg</t>
         </is>
       </c>
       <c r="B102" s="11" t="inlineStr">
         <is>
-          <t>logos</t>
+          <t>images</t>
         </is>
       </c>
       <c r="C102" s="11" t="inlineStr">
         <is>
-          <t>SVG</t>
+          <t>JPEG</t>
         </is>
       </c>
       <c r="D102" s="11" t="inlineStr">
         <is>
-          <t>20.2 KB</t>
+          <t>418.9 KB</t>
         </is>
       </c>
       <c r="E102" s="12" t="inlineStr">
         <is>
-          <t>Logo asset — logo_grey</t>
+          <t>Photography / imagery asset</t>
         </is>
       </c>
     </row>
     <row r="103" ht="16" customHeight="1">
       <c r="A103" s="9" t="inlineStr">
         <is>
-          <t>logos/logo_white.png</t>
+          <t>images/slides/shutterstock_1510566293_RoyalWelshbrug_zwart_1920x1280px_dark-2x1.jpg</t>
         </is>
       </c>
       <c r="B103" s="9" t="inlineStr">
         <is>
-          <t>logos</t>
+          <t>images</t>
         </is>
       </c>
       <c r="C103" s="9" t="inlineStr">
         <is>
-          <t>PNG</t>
+          <t>JPEG</t>
         </is>
       </c>
       <c r="D103" s="9" t="inlineStr">
         <is>
-          <t>8.4 KB</t>
+          <t>635.9 KB</t>
         </is>
       </c>
       <c r="E103" s="10" t="inlineStr">
         <is>
-          <t>Logo asset — logo_white</t>
+          <t>Photography / imagery asset</t>
         </is>
       </c>
     </row>
     <row r="104" ht="16" customHeight="1">
       <c r="A104" s="11" t="inlineStr">
         <is>
-          <t>messaging/audiences.json</t>
+          <t>logos/apple-touch-icon-180.png</t>
         </is>
       </c>
       <c r="B104" s="11" t="inlineStr">
         <is>
-          <t>messaging</t>
+          <t>logos</t>
         </is>
       </c>
       <c r="C104" s="11" t="inlineStr">
         <is>
-          <t>JSON</t>
+          <t>PNG</t>
         </is>
       </c>
       <c r="D104" s="11" t="inlineStr">
         <is>
-          <t>10.8 KB</t>
+          <t>18.5 KB</t>
         </is>
       </c>
       <c r="E104" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Logo asset — apple-touch-icon-180</t>
         </is>
       </c>
     </row>
     <row r="105" ht="16" customHeight="1">
       <c r="A105" s="9" t="inlineStr">
         <is>
-          <t>messaging/narratives.json</t>
+          <t>logos/favicon-192.png</t>
         </is>
       </c>
       <c r="B105" s="9" t="inlineStr">
         <is>
-          <t>messaging</t>
+          <t>logos</t>
         </is>
       </c>
       <c r="C105" s="9" t="inlineStr">
         <is>
-          <t>JSON</t>
+          <t>PNG</t>
         </is>
       </c>
       <c r="D105" s="9" t="inlineStr">
         <is>
-          <t>6.6 KB</t>
+          <t>20.4 KB</t>
         </is>
       </c>
       <c r="E105" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Logo asset — favicon-192</t>
         </is>
       </c>
     </row>
     <row r="106" ht="16" customHeight="1">
       <c r="A106" s="11" t="inlineStr">
         <is>
-          <t>messaging/pillars.json</t>
+          <t>logos/favicon-32.png</t>
         </is>
       </c>
       <c r="B106" s="11" t="inlineStr">
         <is>
-          <t>messaging</t>
+          <t>logos</t>
         </is>
       </c>
       <c r="C106" s="11" t="inlineStr">
         <is>
-          <t>JSON</t>
+          <t>PNG</t>
         </is>
       </c>
       <c r="D106" s="11" t="inlineStr">
         <is>
-          <t>5.9 KB</t>
+          <t>1.1 KB</t>
         </is>
       </c>
       <c r="E106" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Logo asset — favicon-32</t>
         </is>
       </c>
     </row>
     <row r="107" ht="16" customHeight="1">
       <c r="A107" s="9" t="inlineStr">
         <is>
-          <t>messaging/proof-points.json</t>
+          <t>logos/favicon.png</t>
         </is>
       </c>
       <c r="B107" s="9" t="inlineStr">
         <is>
-          <t>messaging</t>
+          <t>logos</t>
         </is>
       </c>
       <c r="C107" s="9" t="inlineStr">
         <is>
-          <t>JSON</t>
+          <t>PNG</t>
         </is>
       </c>
       <c r="D107" s="9" t="inlineStr">
         <is>
-          <t>6.8 KB</t>
+          <t>35.2 KB</t>
         </is>
       </c>
       <c r="E107" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Logo asset — favicon</t>
         </is>
       </c>
     </row>
     <row r="108" ht="16" customHeight="1">
       <c r="A108" s="11" t="inlineStr">
         <is>
-          <t>people.json</t>
+          <t>logos/logo.png</t>
         </is>
       </c>
       <c r="B108" s="11" t="inlineStr">
         <is>
-          <t>root</t>
+          <t>logos</t>
         </is>
       </c>
       <c r="C108" s="11" t="inlineStr">
         <is>
-          <t>JSON</t>
+          <t>PNG</t>
         </is>
       </c>
       <c r="D108" s="11" t="inlineStr">
         <is>
-          <t>1.2 KB</t>
+          <t>23.2 KB</t>
         </is>
       </c>
       <c r="E108" s="12" t="inlineStr">
         <is>
-          <t>Named contacts / key people roster</t>
+          <t>Logo asset — logo</t>
         </is>
       </c>
     </row>
     <row r="109" ht="16" customHeight="1">
       <c r="A109" s="9" t="inlineStr">
         <is>
-          <t>press-releases/approval-matrix.json</t>
+          <t>logos/logo.svg</t>
         </is>
       </c>
       <c r="B109" s="9" t="inlineStr">
         <is>
-          <t>press-releases</t>
+          <t>logos</t>
         </is>
       </c>
       <c r="C109" s="9" t="inlineStr">
         <is>
-          <t>JSON</t>
+          <t>SVG</t>
         </is>
       </c>
       <c r="D109" s="9" t="inlineStr">
         <is>
-          <t>1.4 KB</t>
+          <t>23.7 KB</t>
         </is>
       </c>
       <c r="E109" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Logo asset — logo</t>
         </is>
       </c>
     </row>
     <row r="110" ht="16" customHeight="1">
       <c r="A110" s="11" t="inlineStr">
         <is>
-          <t>press-releases/boilerplate.json</t>
+          <t>logos/logo_grey.svg</t>
         </is>
       </c>
       <c r="B110" s="11" t="inlineStr">
         <is>
-          <t>press-releases</t>
+          <t>logos</t>
         </is>
       </c>
       <c r="C110" s="11" t="inlineStr">
         <is>
-          <t>JSON</t>
+          <t>SVG</t>
         </is>
       </c>
       <c r="D110" s="11" t="inlineStr">
         <is>
-          <t>1.9 KB</t>
+          <t>20.2 KB</t>
         </is>
       </c>
       <c r="E110" s="12" t="inlineStr">
         <is>
-          <t>Reusable legal/footer text snippets</t>
+          <t>Logo asset — logo_grey</t>
         </is>
       </c>
     </row>
     <row r="111" ht="16" customHeight="1">
       <c r="A111" s="9" t="inlineStr">
         <is>
-          <t>press-releases/distribution-lists.json</t>
+          <t>logos/logo_white.png</t>
         </is>
       </c>
       <c r="B111" s="9" t="inlineStr">
         <is>
-          <t>press-releases</t>
+          <t>logos</t>
         </is>
       </c>
       <c r="C111" s="9" t="inlineStr">
         <is>
-          <t>JSON</t>
+          <t>PNG</t>
         </is>
       </c>
       <c r="D111" s="9" t="inlineStr">
         <is>
-          <t>2.1 KB</t>
+          <t>8.4 KB</t>
         </is>
       </c>
       <c r="E111" s="10" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Logo asset — logo_white</t>
         </is>
       </c>
     </row>
     <row r="112" ht="16" customHeight="1">
       <c r="A112" s="11" t="inlineStr">
         <is>
-          <t>press-releases/spokespersons.json</t>
+          <t>messaging/audiences.json</t>
         </is>
       </c>
       <c r="B112" s="11" t="inlineStr">
         <is>
-          <t>press-releases</t>
+          <t>messaging</t>
         </is>
       </c>
       <c r="C112" s="11" t="inlineStr">
@@ -3787,7 +3793,7 @@
       </c>
       <c r="D112" s="11" t="inlineStr">
         <is>
-          <t>3.5 KB</t>
+          <t>10.8 KB</t>
         </is>
       </c>
       <c r="E112" s="12" t="inlineStr">
@@ -3799,12 +3805,12 @@
     <row r="113" ht="16" customHeight="1">
       <c r="A113" s="9" t="inlineStr">
         <is>
-          <t>profile.json</t>
+          <t>messaging/narratives.json</t>
         </is>
       </c>
       <c r="B113" s="9" t="inlineStr">
         <is>
-          <t>root</t>
+          <t>messaging</t>
         </is>
       </c>
       <c r="C113" s="9" t="inlineStr">
@@ -3814,24 +3820,24 @@
       </c>
       <c r="D113" s="9" t="inlineStr">
         <is>
-          <t>8.0 KB</t>
+          <t>6.6 KB</t>
         </is>
       </c>
       <c r="E113" s="10" t="inlineStr">
         <is>
-          <t>Company profile — description, services, legal identity</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="114" ht="16" customHeight="1">
       <c r="A114" s="11" t="inlineStr">
         <is>
-          <t>proposals/boilerplate.json</t>
+          <t>messaging/pillars.json</t>
         </is>
       </c>
       <c r="B114" s="11" t="inlineStr">
         <is>
-          <t>proposals</t>
+          <t>messaging</t>
         </is>
       </c>
       <c r="C114" s="11" t="inlineStr">
@@ -3841,24 +3847,24 @@
       </c>
       <c r="D114" s="11" t="inlineStr">
         <is>
-          <t>4.3 KB</t>
+          <t>5.9 KB</t>
         </is>
       </c>
       <c r="E114" s="12" t="inlineStr">
         <is>
-          <t>Reusable legal/footer text snippets</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="115" ht="16" customHeight="1">
       <c r="A115" s="9" t="inlineStr">
         <is>
-          <t>proposals/case-studies.json</t>
+          <t>messaging/proof-points.json</t>
         </is>
       </c>
       <c r="B115" s="9" t="inlineStr">
         <is>
-          <t>proposals</t>
+          <t>messaging</t>
         </is>
       </c>
       <c r="C115" s="9" t="inlineStr">
@@ -3868,7 +3874,7 @@
       </c>
       <c r="D115" s="9" t="inlineStr">
         <is>
-          <t>18.5 KB</t>
+          <t>6.8 KB</t>
         </is>
       </c>
       <c r="E115" s="10" t="inlineStr">
@@ -3880,12 +3886,12 @@
     <row r="116" ht="16" customHeight="1">
       <c r="A116" s="11" t="inlineStr">
         <is>
-          <t>proposals/differentiators.json</t>
+          <t>people.json</t>
         </is>
       </c>
       <c r="B116" s="11" t="inlineStr">
         <is>
-          <t>proposals</t>
+          <t>root</t>
         </is>
       </c>
       <c r="C116" s="11" t="inlineStr">
@@ -3895,24 +3901,24 @@
       </c>
       <c r="D116" s="11" t="inlineStr">
         <is>
-          <t>4.2 KB</t>
+          <t>1.2 KB</t>
         </is>
       </c>
       <c r="E116" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Named contacts / key people roster</t>
         </is>
       </c>
     </row>
     <row r="117" ht="16" customHeight="1">
       <c r="A117" s="9" t="inlineStr">
         <is>
-          <t>proposals/methodologies.json</t>
+          <t>press-releases/approval-matrix.json</t>
         </is>
       </c>
       <c r="B117" s="9" t="inlineStr">
         <is>
-          <t>proposals</t>
+          <t>press-releases</t>
         </is>
       </c>
       <c r="C117" s="9" t="inlineStr">
@@ -3922,7 +3928,7 @@
       </c>
       <c r="D117" s="9" t="inlineStr">
         <is>
-          <t>4.5 KB</t>
+          <t>1.4 KB</t>
         </is>
       </c>
       <c r="E117" s="10" t="inlineStr">
@@ -3934,12 +3940,12 @@
     <row r="118" ht="16" customHeight="1">
       <c r="A118" s="11" t="inlineStr">
         <is>
-          <t>proposals/partnerships.json</t>
+          <t>press-releases/boilerplate.json</t>
         </is>
       </c>
       <c r="B118" s="11" t="inlineStr">
         <is>
-          <t>proposals</t>
+          <t>press-releases</t>
         </is>
       </c>
       <c r="C118" s="11" t="inlineStr">
@@ -3949,24 +3955,24 @@
       </c>
       <c r="D118" s="11" t="inlineStr">
         <is>
-          <t>1.0 KB</t>
+          <t>1.9 KB</t>
         </is>
       </c>
       <c r="E118" s="12" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Reusable legal/footer text snippets</t>
         </is>
       </c>
     </row>
     <row r="119" ht="16" customHeight="1">
       <c r="A119" s="9" t="inlineStr">
         <is>
-          <t>proposals/team-bios.json</t>
+          <t>press-releases/distribution-lists.json</t>
         </is>
       </c>
       <c r="B119" s="9" t="inlineStr">
         <is>
-          <t>proposals</t>
+          <t>press-releases</t>
         </is>
       </c>
       <c r="C119" s="9" t="inlineStr">
@@ -3976,7 +3982,7 @@
       </c>
       <c r="D119" s="9" t="inlineStr">
         <is>
-          <t>9.7 KB</t>
+          <t>2.1 KB</t>
         </is>
       </c>
       <c r="E119" s="10" t="inlineStr">
@@ -3988,12 +3994,12 @@
     <row r="120" ht="16" customHeight="1">
       <c r="A120" s="11" t="inlineStr">
         <is>
-          <t>proposals/testimonials.json</t>
+          <t>press-releases/spokespersons.json</t>
         </is>
       </c>
       <c r="B120" s="11" t="inlineStr">
         <is>
-          <t>proposals</t>
+          <t>press-releases</t>
         </is>
       </c>
       <c r="C120" s="11" t="inlineStr">
@@ -4003,7 +4009,7 @@
       </c>
       <c r="D120" s="11" t="inlineStr">
         <is>
-          <t>2.0 KB</t>
+          <t>3.5 KB</t>
         </is>
       </c>
       <c r="E120" s="12" t="inlineStr">
@@ -4015,141 +4021,357 @@
     <row r="121" ht="16" customHeight="1">
       <c r="A121" s="9" t="inlineStr">
         <is>
-          <t>templates/docx/Duke-Strategies-Letterhead.docx</t>
+          <t>profile.json</t>
         </is>
       </c>
       <c r="B121" s="9" t="inlineStr">
         <is>
-          <t>templates</t>
+          <t>root</t>
         </is>
       </c>
       <c r="C121" s="9" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>JSON</t>
         </is>
       </c>
       <c r="D121" s="9" t="inlineStr">
         <is>
-          <t>46.1 KB</t>
+          <t>8.4 KB</t>
         </is>
       </c>
       <c r="E121" s="10" t="inlineStr">
         <is>
-          <t>Branded Word styles template</t>
+          <t>Company profile — description, services, legal identity</t>
         </is>
       </c>
     </row>
     <row r="122" ht="16" customHeight="1">
       <c r="A122" s="11" t="inlineStr">
         <is>
-          <t>templates/docx/Duke-Strategies-Report.docx</t>
+          <t>proposals/boilerplate.json</t>
         </is>
       </c>
       <c r="B122" s="11" t="inlineStr">
         <is>
-          <t>templates</t>
+          <t>proposals</t>
         </is>
       </c>
       <c r="C122" s="11" t="inlineStr">
         <is>
-          <t>DOCX</t>
+          <t>JSON</t>
         </is>
       </c>
       <c r="D122" s="11" t="inlineStr">
         <is>
-          <t>216.9 KB</t>
+          <t>4.3 KB</t>
         </is>
       </c>
       <c r="E122" s="12" t="inlineStr">
         <is>
-          <t>Branded Word styles template</t>
+          <t>Reusable legal/footer text snippets</t>
         </is>
       </c>
     </row>
     <row r="123" ht="16" customHeight="1">
       <c r="A123" s="9" t="inlineStr">
         <is>
-          <t>templates/html/business-cards.html</t>
+          <t>proposals/case-studies.json</t>
         </is>
       </c>
       <c r="B123" s="9" t="inlineStr">
         <is>
-          <t>templates</t>
+          <t>proposals</t>
         </is>
       </c>
       <c r="C123" s="9" t="inlineStr">
         <is>
-          <t>HTML</t>
+          <t>JSON</t>
         </is>
       </c>
       <c r="D123" s="9" t="inlineStr">
         <is>
-          <t>20.0 KB</t>
+          <t>18.5 KB</t>
         </is>
       </c>
       <c r="E123" s="10" t="inlineStr">
         <is>
-          <t>Branded HTML template</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="124" ht="16" customHeight="1">
       <c r="A124" s="11" t="inlineStr">
         <is>
-          <t>templates/html/email-signatures.html</t>
+          <t>proposals/differentiators.json</t>
         </is>
       </c>
       <c r="B124" s="11" t="inlineStr">
         <is>
-          <t>templates</t>
+          <t>proposals</t>
         </is>
       </c>
       <c r="C124" s="11" t="inlineStr">
         <is>
-          <t>HTML</t>
+          <t>JSON</t>
         </is>
       </c>
       <c r="D124" s="11" t="inlineStr">
         <is>
-          <t>21.8 KB</t>
+          <t>4.2 KB</t>
         </is>
       </c>
       <c r="E124" s="12" t="inlineStr">
         <is>
-          <t>Branded HTML template</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="125" ht="16" customHeight="1">
       <c r="A125" s="9" t="inlineStr">
         <is>
+          <t>proposals/methodologies.json</t>
+        </is>
+      </c>
+      <c r="B125" s="9" t="inlineStr">
+        <is>
+          <t>proposals</t>
+        </is>
+      </c>
+      <c r="C125" s="9" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+      <c r="D125" s="9" t="inlineStr">
+        <is>
+          <t>4.5 KB</t>
+        </is>
+      </c>
+      <c r="E125" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="16" customHeight="1">
+      <c r="A126" s="11" t="inlineStr">
+        <is>
+          <t>proposals/partnerships.json</t>
+        </is>
+      </c>
+      <c r="B126" s="11" t="inlineStr">
+        <is>
+          <t>proposals</t>
+        </is>
+      </c>
+      <c r="C126" s="11" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+      <c r="D126" s="11" t="inlineStr">
+        <is>
+          <t>1.0 KB</t>
+        </is>
+      </c>
+      <c r="E126" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="16" customHeight="1">
+      <c r="A127" s="9" t="inlineStr">
+        <is>
+          <t>proposals/team-bios.json</t>
+        </is>
+      </c>
+      <c r="B127" s="9" t="inlineStr">
+        <is>
+          <t>proposals</t>
+        </is>
+      </c>
+      <c r="C127" s="9" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+      <c r="D127" s="9" t="inlineStr">
+        <is>
+          <t>9.7 KB</t>
+        </is>
+      </c>
+      <c r="E127" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="16" customHeight="1">
+      <c r="A128" s="11" t="inlineStr">
+        <is>
+          <t>proposals/testimonials.json</t>
+        </is>
+      </c>
+      <c r="B128" s="11" t="inlineStr">
+        <is>
+          <t>proposals</t>
+        </is>
+      </c>
+      <c r="C128" s="11" t="inlineStr">
+        <is>
+          <t>JSON</t>
+        </is>
+      </c>
+      <c r="D128" s="11" t="inlineStr">
+        <is>
+          <t>2.0 KB</t>
+        </is>
+      </c>
+      <c r="E128" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="16" customHeight="1">
+      <c r="A129" s="9" t="inlineStr">
+        <is>
+          <t>templates/docx/Duke-Strategies-Letterhead.docx</t>
+        </is>
+      </c>
+      <c r="B129" s="9" t="inlineStr">
+        <is>
+          <t>templates</t>
+        </is>
+      </c>
+      <c r="C129" s="9" t="inlineStr">
+        <is>
+          <t>DOCX</t>
+        </is>
+      </c>
+      <c r="D129" s="9" t="inlineStr">
+        <is>
+          <t>46.1 KB</t>
+        </is>
+      </c>
+      <c r="E129" s="10" t="inlineStr">
+        <is>
+          <t>Branded Word styles template</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="16" customHeight="1">
+      <c r="A130" s="11" t="inlineStr">
+        <is>
+          <t>templates/docx/Duke-Strategies-Report.docx</t>
+        </is>
+      </c>
+      <c r="B130" s="11" t="inlineStr">
+        <is>
+          <t>templates</t>
+        </is>
+      </c>
+      <c r="C130" s="11" t="inlineStr">
+        <is>
+          <t>DOCX</t>
+        </is>
+      </c>
+      <c r="D130" s="11" t="inlineStr">
+        <is>
+          <t>216.9 KB</t>
+        </is>
+      </c>
+      <c r="E130" s="12" t="inlineStr">
+        <is>
+          <t>Branded Word styles template</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="16" customHeight="1">
+      <c r="A131" s="9" t="inlineStr">
+        <is>
+          <t>templates/html/business-cards.html</t>
+        </is>
+      </c>
+      <c r="B131" s="9" t="inlineStr">
+        <is>
+          <t>templates</t>
+        </is>
+      </c>
+      <c r="C131" s="9" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="D131" s="9" t="inlineStr">
+        <is>
+          <t>20.0 KB</t>
+        </is>
+      </c>
+      <c r="E131" s="10" t="inlineStr">
+        <is>
+          <t>Branded HTML template</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="16" customHeight="1">
+      <c r="A132" s="11" t="inlineStr">
+        <is>
+          <t>templates/html/email-signatures.html</t>
+        </is>
+      </c>
+      <c r="B132" s="11" t="inlineStr">
+        <is>
+          <t>templates</t>
+        </is>
+      </c>
+      <c r="C132" s="11" t="inlineStr">
+        <is>
+          <t>HTML</t>
+        </is>
+      </c>
+      <c r="D132" s="11" t="inlineStr">
+        <is>
+          <t>21.8 KB</t>
+        </is>
+      </c>
+      <c r="E132" s="12" t="inlineStr">
+        <is>
+          <t>Branded HTML template</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="16" customHeight="1">
+      <c r="A133" s="9" t="inlineStr">
+        <is>
           <t>tokens.css</t>
         </is>
       </c>
-      <c r="B125" s="9" t="inlineStr">
+      <c r="B133" s="9" t="inlineStr">
         <is>
           <t>root</t>
         </is>
       </c>
-      <c r="C125" s="9" t="inlineStr">
+      <c r="C133" s="9" t="inlineStr">
         <is>
           <t>CSS</t>
         </is>
       </c>
-      <c r="D125" s="9" t="inlineStr">
-        <is>
-          <t>18.2 KB</t>
-        </is>
-      </c>
-      <c r="E125" s="10" t="inlineStr">
+      <c r="D133" s="9" t="inlineStr">
+        <is>
+          <t>18.4 KB</t>
+        </is>
+      </c>
+      <c r="E133" s="10" t="inlineStr">
         <is>
           <t>CSS design tokens mapping brand colors to CSS variables</t>
         </is>
       </c>
     </row>
-    <row r="126" ht="8" customHeight="1"/>
-    <row r="127">
-      <c r="A127" s="7" t="inlineStr">
+    <row r="134" ht="8" customHeight="1"/>
+    <row r="135">
+      <c r="A135" s="7" t="inlineStr">
         <is>
           <t>Duke Strategies  ·  Confidential — Not for distribution</t>
         </is>
@@ -4157,7 +4379,7 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A127:F127"/>
+    <mergeCell ref="A135:F135"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4242,12 +4464,12 @@
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>#FF7F66</t>
+          <t>#222222</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>rgb(255, 127, 102)</t>
+          <t>rgb(34, 34, 34)</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
@@ -4269,12 +4491,12 @@
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>#DFDFE0</t>
+          <t>#5A595C</t>
         </is>
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>rgb(223, 223, 224)</t>
+          <t>rgb(90, 89, 92)</t>
         </is>
       </c>
       <c r="E6" s="17" t="inlineStr">
@@ -4296,12 +4518,12 @@
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>#F47E6C</t>
+          <t>#FF7F66</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
         <is>
-          <t>rgb(244, 126, 108)</t>
+          <t>rgb(255, 127, 102)</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
@@ -4323,161 +4545,161 @@
       </c>
       <c r="C8" s="16" t="inlineStr">
         <is>
+          <t>#3A393C</t>
+        </is>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>rgb(58, 57, 60)</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="inlineStr">
+        <is>
+          <t>Main body text</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   </t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>Textlight</t>
+        </is>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
           <t>#807F83</t>
         </is>
       </c>
-      <c r="D8" s="16" t="inlineStr">
+      <c r="D9" s="14" t="inlineStr">
         <is>
           <t>rgb(128, 127, 131)</t>
         </is>
       </c>
-      <c r="E8" s="17" t="inlineStr">
-        <is>
-          <t>Main body text</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="E9" s="15" t="inlineStr">
+        <is>
+          <t>Captions, footers, secondary labels</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">   </t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>Textlight</t>
-        </is>
-      </c>
-      <c r="C9" s="14" t="inlineStr">
-        <is>
-          <t>#DFDFE0</t>
-        </is>
-      </c>
-      <c r="D9" s="14" t="inlineStr">
-        <is>
-          <t>rgb(223, 223, 224)</t>
-        </is>
-      </c>
-      <c r="E9" s="15" t="inlineStr">
-        <is>
-          <t>Captions, footers, secondary labels</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="20" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>Background</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>#FFFFFF</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>rgb(255, 255, 255)</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="inlineStr">
+        <is>
+          <t>Page / sheet background</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">   </t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
-        <is>
-          <t>Background</t>
-        </is>
-      </c>
-      <c r="C10" s="16" t="inlineStr">
-        <is>
-          <t>#FFFFFF</t>
-        </is>
-      </c>
-      <c r="D10" s="16" t="inlineStr">
-        <is>
-          <t>rgb(255, 255, 255)</t>
-        </is>
-      </c>
-      <c r="E10" s="17" t="inlineStr">
-        <is>
-          <t>Page / sheet background</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>Success</t>
+        </is>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>#5B9A6B</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="inlineStr">
+        <is>
+          <t>rgb(91, 154, 107)</t>
+        </is>
+      </c>
+      <c r="E11" s="15" t="inlineStr">
+        <is>
+          <t>Success / positive state</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">   </t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
-        <is>
-          <t>Success</t>
-        </is>
-      </c>
-      <c r="C11" s="14" t="inlineStr">
-        <is>
-          <t>#4CAF50</t>
-        </is>
-      </c>
-      <c r="D11" s="14" t="inlineStr">
-        <is>
-          <t>rgb(76, 175, 80)</t>
-        </is>
-      </c>
-      <c r="E11" s="15" t="inlineStr">
-        <is>
-          <t>Success / positive state</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="22" t="inlineStr">
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="C12" s="16" t="inlineStr">
+        <is>
+          <t>#D4A544</t>
+        </is>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>rgb(212, 165, 68)</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>Warning / caution state</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">   </t>
         </is>
       </c>
-      <c r="B12" s="16" t="inlineStr">
-        <is>
-          <t>Warning</t>
-        </is>
-      </c>
-      <c r="C12" s="16" t="inlineStr">
-        <is>
-          <t>#FFC107</t>
-        </is>
-      </c>
-      <c r="D12" s="16" t="inlineStr">
-        <is>
-          <t>rgb(255, 193, 7)</t>
-        </is>
-      </c>
-      <c r="E12" s="17" t="inlineStr">
-        <is>
-          <t>Warning / caution state</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="23" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>Error</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>#C4544A</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>rgb(196, 84, 74)</t>
+        </is>
+      </c>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>Error / danger state</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">   </t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
-        <is>
-          <t>Error</t>
-        </is>
-      </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>#DC3545</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="inlineStr">
-        <is>
-          <t>rgb(220, 53, 69)</t>
-        </is>
-      </c>
-      <c r="E13" s="15" t="inlineStr">
-        <is>
-          <t>Error / danger state</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   </t>
-        </is>
-      </c>
       <c r="B14" s="16" t="inlineStr">
         <is>
           <t>Accenthover</t>
@@ -4485,12 +4707,12 @@
       </c>
       <c r="C14" s="16" t="inlineStr">
         <is>
-          <t>#EE5536</t>
+          <t>#E86B54</t>
         </is>
       </c>
       <c r="D14" s="16" t="inlineStr">
         <is>
-          <t>rgb(238, 85, 54)</t>
+          <t>rgb(232, 107, 84)</t>
         </is>
       </c>
       <c r="E14" s="17" t="inlineStr">
@@ -4500,7 +4722,7 @@
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="25" t="inlineStr">
+      <c r="A15" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">   </t>
         </is>
@@ -4616,7 +4838,7 @@
       <c r="F4" s="3" t="n"/>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="26" t="inlineStr">
+      <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Heading</t>
         </is>
@@ -4648,7 +4870,7 @@
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="27" t="inlineStr">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>Body</t>
         </is>
@@ -4680,7 +4902,7 @@
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="27" t="inlineStr">
         <is>
           <t>Mono</t>
         </is>
@@ -4763,7 +4985,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -4824,7 +5046,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>0.55</t>
+          <t>0.5</t>
         </is>
       </c>
     </row>
@@ -5009,9 +5231,169 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="8" customHeight="1"/>
-    <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="9" t="inlineStr">
+        <is>
+          <t>images/erasmus-bridge-rotterdam-grayscale.jpg</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="inlineStr">
+        <is>
+          <t>cover, closing</t>
+        </is>
+      </c>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F15" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>images/cable-bridge-grayscale-dramatic.jpg</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>cover, divider</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>images/modern-bridge-bw-dramatic.jpg</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="inlineStr">
+        <is>
+          <t>cover, divider</t>
+        </is>
+      </c>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>images/bridge-fog-water-minimalist.jpg</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>divider, closing</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>images/modern-cable-bridge-calm-water.jpg</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="inlineStr">
+        <is>
+          <t>divider, background</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="8" customHeight="1"/>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>Duke Strategies  ·  Confidential — Not for distribution</t>
         </is>
@@ -5020,7 +5402,7 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A21:F21"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5220,7 +5602,7 @@
       <c r="E19" s="3" t="n"/>
     </row>
     <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="26" t="inlineStr">
+      <c r="A20" s="27" t="inlineStr">
         <is>
           <t>Strategic Advisory</t>
         </is>
@@ -5247,7 +5629,7 @@
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="27" t="inlineStr">
+      <c r="A21" s="28" t="inlineStr">
         <is>
           <t>Crisis Communications</t>
         </is>
@@ -5274,7 +5656,7 @@
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="26" t="inlineStr">
+      <c r="A22" s="27" t="inlineStr">
         <is>
           <t>Stakeholder Mapping &amp; Engagement</t>
         </is>
@@ -5301,7 +5683,7 @@
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="27" t="inlineStr">
+      <c r="A23" s="28" t="inlineStr">
         <is>
           <t>M&amp;A Communications</t>
         </is>
@@ -5328,7 +5710,7 @@
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="26" t="inlineStr">
+      <c r="A24" s="27" t="inlineStr">
         <is>
           <t>Media Training &amp; Positioning</t>
         </is>
@@ -5355,7 +5737,7 @@
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="27" t="inlineStr">
+      <c r="A25" s="28" t="inlineStr">
         <is>
           <t>Change Management Communications</t>
         </is>
@@ -5382,7 +5764,7 @@
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="26" t="inlineStr">
+      <c r="A26" s="27" t="inlineStr">
         <is>
           <t>Issue Management</t>
         </is>
@@ -5495,7 +5877,7 @@
       <c r="E4" s="3" t="n"/>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="26" t="inlineStr">
+      <c r="A5" s="27" t="inlineStr">
         <is>
           <t>Ingo Heijnen</t>
         </is>
@@ -5522,7 +5904,7 @@
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="27" t="inlineStr">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>Arien Stuijt</t>
         </is>
@@ -5549,7 +5931,7 @@
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="27" t="inlineStr">
         <is>
           <t>Emma van Gelder</t>
         </is>
@@ -5576,7 +5958,7 @@
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="27" t="inlineStr">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>William Masquelier</t>
         </is>
@@ -5603,7 +5985,7 @@
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="26" t="inlineStr">
+      <c r="A9" s="27" t="inlineStr">
         <is>
           <t>Bas van 't Wout</t>
         </is>
@@ -5630,7 +6012,7 @@
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="27" t="inlineStr">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t>Pieter Cobelens</t>
         </is>

</xml_diff>